<commit_message>
add the protein classification leaves and refresh the root roll-up and spec curve
</commit_message>
<xml_diff>
--- a/04_Figures/02_classification/c_data/results.xlsx
+++ b/04_Figures/02_classification/c_data/results.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">level</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t xml:space="preserve">pathways</t>
+  </si>
+  <si>
+    <t xml:space="preserve">proteins</t>
   </si>
 </sst>
 </file>
@@ -8379,6 +8382,3730 @@
         <v>0.261857529826539</v>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="s">
+        <v>31</v>
+      </c>
+      <c r="B210" t="s">
+        <v>14</v>
+      </c>
+      <c r="C210" t="s">
+        <v>15</v>
+      </c>
+      <c r="D210" t="s">
+        <v>16</v>
+      </c>
+      <c r="E210" t="n">
+        <v>15</v>
+      </c>
+      <c r="F210" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G210" t="n">
+        <v>0</v>
+      </c>
+      <c r="H210" t="n">
+        <v>0</v>
+      </c>
+      <c r="I210" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" t="n">
+        <v>0</v>
+      </c>
+      <c r="K210"/>
+      <c r="L210"/>
+      <c r="M210"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="s">
+        <v>31</v>
+      </c>
+      <c r="B211" t="s">
+        <v>14</v>
+      </c>
+      <c r="C211" t="s">
+        <v>15</v>
+      </c>
+      <c r="D211" t="s">
+        <v>16</v>
+      </c>
+      <c r="E211" t="n">
+        <v>15</v>
+      </c>
+      <c r="F211" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G211" t="n">
+        <v>200</v>
+      </c>
+      <c r="H211" t="n">
+        <v>0</v>
+      </c>
+      <c r="I211" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" t="n">
+        <v>0</v>
+      </c>
+      <c r="K211" t="n">
+        <v>1</v>
+      </c>
+      <c r="L211" t="n">
+        <v>0.0990178571428572</v>
+      </c>
+      <c r="M211" t="n">
+        <v>0.208369802896195</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="s">
+        <v>31</v>
+      </c>
+      <c r="B212" t="s">
+        <v>14</v>
+      </c>
+      <c r="C212" t="s">
+        <v>17</v>
+      </c>
+      <c r="D212" t="s">
+        <v>16</v>
+      </c>
+      <c r="E212" t="n">
+        <v>15</v>
+      </c>
+      <c r="F212" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G212" t="n">
+        <v>0</v>
+      </c>
+      <c r="H212" t="n">
+        <v>0</v>
+      </c>
+      <c r="I212" t="n">
+        <v>0</v>
+      </c>
+      <c r="J212" t="n">
+        <v>0</v>
+      </c>
+      <c r="K212"/>
+      <c r="L212"/>
+      <c r="M212"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="s">
+        <v>31</v>
+      </c>
+      <c r="B213" t="s">
+        <v>14</v>
+      </c>
+      <c r="C213" t="s">
+        <v>17</v>
+      </c>
+      <c r="D213" t="s">
+        <v>16</v>
+      </c>
+      <c r="E213" t="n">
+        <v>15</v>
+      </c>
+      <c r="F213" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G213" t="n">
+        <v>200</v>
+      </c>
+      <c r="H213" t="n">
+        <v>0</v>
+      </c>
+      <c r="I213" t="n">
+        <v>0</v>
+      </c>
+      <c r="J213" t="n">
+        <v>0</v>
+      </c>
+      <c r="K213" t="n">
+        <v>1</v>
+      </c>
+      <c r="L213" t="n">
+        <v>0.111875</v>
+      </c>
+      <c r="M213" t="n">
+        <v>0.221821588521361</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="s">
+        <v>31</v>
+      </c>
+      <c r="B214" t="s">
+        <v>14</v>
+      </c>
+      <c r="C214" t="s">
+        <v>18</v>
+      </c>
+      <c r="D214" t="s">
+        <v>16</v>
+      </c>
+      <c r="E214" t="n">
+        <v>15</v>
+      </c>
+      <c r="F214" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G214" t="n">
+        <v>0</v>
+      </c>
+      <c r="H214" t="n">
+        <v>0.214285714285714</v>
+      </c>
+      <c r="I214" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" t="n">
+        <v>0.498005719950453</v>
+      </c>
+      <c r="K214"/>
+      <c r="L214"/>
+      <c r="M214"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="s">
+        <v>31</v>
+      </c>
+      <c r="B215" t="s">
+        <v>14</v>
+      </c>
+      <c r="C215" t="s">
+        <v>18</v>
+      </c>
+      <c r="D215" t="s">
+        <v>16</v>
+      </c>
+      <c r="E215" t="n">
+        <v>15</v>
+      </c>
+      <c r="F215" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G215" t="n">
+        <v>200</v>
+      </c>
+      <c r="H215" t="n">
+        <v>0.214285714285714</v>
+      </c>
+      <c r="I215" t="n">
+        <v>0</v>
+      </c>
+      <c r="J215" t="n">
+        <v>0.498005719950453</v>
+      </c>
+      <c r="K215" t="n">
+        <v>0.462686567164179</v>
+      </c>
+      <c r="L215" t="n">
+        <v>0.245357142857143</v>
+      </c>
+      <c r="M215" t="n">
+        <v>0.2395803170871</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="s">
+        <v>31</v>
+      </c>
+      <c r="B216" t="s">
+        <v>14</v>
+      </c>
+      <c r="C216" t="s">
+        <v>20</v>
+      </c>
+      <c r="D216" t="s">
+        <v>16</v>
+      </c>
+      <c r="E216" t="n">
+        <v>15</v>
+      </c>
+      <c r="F216" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G216" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" t="n">
+        <v>0.392857142857143</v>
+      </c>
+      <c r="I216" t="n">
+        <v>0.0632927713151577</v>
+      </c>
+      <c r="J216" t="n">
+        <v>0.722421514399128</v>
+      </c>
+      <c r="K216"/>
+      <c r="L216"/>
+      <c r="M216"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="s">
+        <v>31</v>
+      </c>
+      <c r="B217" t="s">
+        <v>14</v>
+      </c>
+      <c r="C217" t="s">
+        <v>20</v>
+      </c>
+      <c r="D217" t="s">
+        <v>16</v>
+      </c>
+      <c r="E217" t="n">
+        <v>15</v>
+      </c>
+      <c r="F217" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G217" t="n">
+        <v>200</v>
+      </c>
+      <c r="H217" t="n">
+        <v>0.392857142857143</v>
+      </c>
+      <c r="I217" t="n">
+        <v>0.0632927713151577</v>
+      </c>
+      <c r="J217" t="n">
+        <v>0.722421514399128</v>
+      </c>
+      <c r="K217" t="n">
+        <v>0.313432835820896</v>
+      </c>
+      <c r="L217" t="n">
+        <v>0.284017857142857</v>
+      </c>
+      <c r="M217" t="n">
+        <v>0.197170314440653</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="s">
+        <v>31</v>
+      </c>
+      <c r="B218" t="s">
+        <v>14</v>
+      </c>
+      <c r="C218" t="s">
+        <v>21</v>
+      </c>
+      <c r="D218" t="s">
+        <v>16</v>
+      </c>
+      <c r="E218" t="n">
+        <v>15</v>
+      </c>
+      <c r="F218" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G218" t="n">
+        <v>0</v>
+      </c>
+      <c r="H218" t="n">
+        <v>0</v>
+      </c>
+      <c r="I218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J218" t="n">
+        <v>0</v>
+      </c>
+      <c r="K218"/>
+      <c r="L218"/>
+      <c r="M218"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="s">
+        <v>31</v>
+      </c>
+      <c r="B219" t="s">
+        <v>14</v>
+      </c>
+      <c r="C219" t="s">
+        <v>21</v>
+      </c>
+      <c r="D219" t="s">
+        <v>16</v>
+      </c>
+      <c r="E219" t="n">
+        <v>15</v>
+      </c>
+      <c r="F219" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G219" t="n">
+        <v>200</v>
+      </c>
+      <c r="H219" t="n">
+        <v>0</v>
+      </c>
+      <c r="I219" t="n">
+        <v>0</v>
+      </c>
+      <c r="J219" t="n">
+        <v>0</v>
+      </c>
+      <c r="K219" t="n">
+        <v>1</v>
+      </c>
+      <c r="L219" t="n">
+        <v>0.00196428571428572</v>
+      </c>
+      <c r="M219" t="n">
+        <v>0.0253671380561481</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="s">
+        <v>31</v>
+      </c>
+      <c r="B220" t="s">
+        <v>14</v>
+      </c>
+      <c r="C220" t="s">
+        <v>22</v>
+      </c>
+      <c r="D220" t="s">
+        <v>16</v>
+      </c>
+      <c r="E220" t="n">
+        <v>15</v>
+      </c>
+      <c r="F220" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G220" t="n">
+        <v>0</v>
+      </c>
+      <c r="H220" t="n">
+        <v>0.392857142857143</v>
+      </c>
+      <c r="I220" t="n">
+        <v>0.0462128719888035</v>
+      </c>
+      <c r="J220" t="n">
+        <v>0.739501413725482</v>
+      </c>
+      <c r="K220"/>
+      <c r="L220"/>
+      <c r="M220"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="s">
+        <v>31</v>
+      </c>
+      <c r="B221" t="s">
+        <v>14</v>
+      </c>
+      <c r="C221" t="s">
+        <v>22</v>
+      </c>
+      <c r="D221" t="s">
+        <v>16</v>
+      </c>
+      <c r="E221" t="n">
+        <v>15</v>
+      </c>
+      <c r="F221" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G221" t="n">
+        <v>200</v>
+      </c>
+      <c r="H221" t="n">
+        <v>0.392857142857143</v>
+      </c>
+      <c r="I221" t="n">
+        <v>0.0462128719888035</v>
+      </c>
+      <c r="J221" t="n">
+        <v>0.739501413725482</v>
+      </c>
+      <c r="K221" t="n">
+        <v>0.562189054726368</v>
+      </c>
+      <c r="L221" t="n">
+        <v>0.424285714285714</v>
+      </c>
+      <c r="M221" t="n">
+        <v>0.232423900781298</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="s">
+        <v>31</v>
+      </c>
+      <c r="B222" t="s">
+        <v>14</v>
+      </c>
+      <c r="C222" t="s">
+        <v>23</v>
+      </c>
+      <c r="D222" t="s">
+        <v>16</v>
+      </c>
+      <c r="E222" t="n">
+        <v>15</v>
+      </c>
+      <c r="F222" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G222" t="n">
+        <v>0</v>
+      </c>
+      <c r="H222" t="n">
+        <v>0.232142857142857</v>
+      </c>
+      <c r="I222" t="n">
+        <v>0</v>
+      </c>
+      <c r="J222" t="n">
+        <v>0.539925007162735</v>
+      </c>
+      <c r="K222"/>
+      <c r="L222"/>
+      <c r="M222"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="s">
+        <v>31</v>
+      </c>
+      <c r="B223" t="s">
+        <v>14</v>
+      </c>
+      <c r="C223" t="s">
+        <v>23</v>
+      </c>
+      <c r="D223" t="s">
+        <v>16</v>
+      </c>
+      <c r="E223" t="n">
+        <v>15</v>
+      </c>
+      <c r="F223" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G223" t="n">
+        <v>200</v>
+      </c>
+      <c r="H223" t="n">
+        <v>0.232142857142857</v>
+      </c>
+      <c r="I223" t="n">
+        <v>0</v>
+      </c>
+      <c r="J223" t="n">
+        <v>0.539925007162735</v>
+      </c>
+      <c r="K223" t="n">
+        <v>0.582089552238806</v>
+      </c>
+      <c r="L223" t="n">
+        <v>0.323839285714286</v>
+      </c>
+      <c r="M223" t="n">
+        <v>0.240024263779417</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s">
+        <v>31</v>
+      </c>
+      <c r="B224" t="s">
+        <v>24</v>
+      </c>
+      <c r="C224" t="s">
+        <v>15</v>
+      </c>
+      <c r="D224" t="s">
+        <v>16</v>
+      </c>
+      <c r="E224" t="n">
+        <v>15</v>
+      </c>
+      <c r="F224" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G224" t="n">
+        <v>0</v>
+      </c>
+      <c r="H224" t="n">
+        <v>0</v>
+      </c>
+      <c r="I224" t="n">
+        <v>0</v>
+      </c>
+      <c r="J224" t="n">
+        <v>0</v>
+      </c>
+      <c r="K224"/>
+      <c r="L224"/>
+      <c r="M224"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="s">
+        <v>31</v>
+      </c>
+      <c r="B225" t="s">
+        <v>24</v>
+      </c>
+      <c r="C225" t="s">
+        <v>15</v>
+      </c>
+      <c r="D225" t="s">
+        <v>16</v>
+      </c>
+      <c r="E225" t="n">
+        <v>15</v>
+      </c>
+      <c r="F225" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G225" t="n">
+        <v>200</v>
+      </c>
+      <c r="H225" t="n">
+        <v>0</v>
+      </c>
+      <c r="I225" t="n">
+        <v>0</v>
+      </c>
+      <c r="J225" t="n">
+        <v>0</v>
+      </c>
+      <c r="K225" t="n">
+        <v>1</v>
+      </c>
+      <c r="L225" t="n">
+        <v>0.101339285714286</v>
+      </c>
+      <c r="M225" t="n">
+        <v>0.234952061537881</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="s">
+        <v>31</v>
+      </c>
+      <c r="B226" t="s">
+        <v>24</v>
+      </c>
+      <c r="C226" t="s">
+        <v>17</v>
+      </c>
+      <c r="D226" t="s">
+        <v>16</v>
+      </c>
+      <c r="E226" t="n">
+        <v>15</v>
+      </c>
+      <c r="F226" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0</v>
+      </c>
+      <c r="H226" t="n">
+        <v>0</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" t="n">
+        <v>0</v>
+      </c>
+      <c r="K226"/>
+      <c r="L226"/>
+      <c r="M226"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="s">
+        <v>31</v>
+      </c>
+      <c r="B227" t="s">
+        <v>24</v>
+      </c>
+      <c r="C227" t="s">
+        <v>17</v>
+      </c>
+      <c r="D227" t="s">
+        <v>16</v>
+      </c>
+      <c r="E227" t="n">
+        <v>15</v>
+      </c>
+      <c r="F227" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G227" t="n">
+        <v>200</v>
+      </c>
+      <c r="H227" t="n">
+        <v>0</v>
+      </c>
+      <c r="I227" t="n">
+        <v>0</v>
+      </c>
+      <c r="J227" t="n">
+        <v>0</v>
+      </c>
+      <c r="K227" t="n">
+        <v>1</v>
+      </c>
+      <c r="L227" t="n">
+        <v>0.102410714285714</v>
+      </c>
+      <c r="M227" t="n">
+        <v>0.227541350833974</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="s">
+        <v>31</v>
+      </c>
+      <c r="B228" t="s">
+        <v>24</v>
+      </c>
+      <c r="C228" t="s">
+        <v>18</v>
+      </c>
+      <c r="D228" t="s">
+        <v>16</v>
+      </c>
+      <c r="E228" t="n">
+        <v>15</v>
+      </c>
+      <c r="F228" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G228" t="n">
+        <v>0</v>
+      </c>
+      <c r="H228" t="n">
+        <v>0</v>
+      </c>
+      <c r="I228" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" t="n">
+        <v>0</v>
+      </c>
+      <c r="K228"/>
+      <c r="L228"/>
+      <c r="M228"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="s">
+        <v>31</v>
+      </c>
+      <c r="B229" t="s">
+        <v>24</v>
+      </c>
+      <c r="C229" t="s">
+        <v>18</v>
+      </c>
+      <c r="D229" t="s">
+        <v>16</v>
+      </c>
+      <c r="E229" t="n">
+        <v>15</v>
+      </c>
+      <c r="F229" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G229" t="n">
+        <v>200</v>
+      </c>
+      <c r="H229" t="n">
+        <v>0</v>
+      </c>
+      <c r="I229" t="n">
+        <v>0</v>
+      </c>
+      <c r="J229" t="n">
+        <v>0</v>
+      </c>
+      <c r="K229" t="n">
+        <v>1</v>
+      </c>
+      <c r="L229" t="n">
+        <v>0.306160714285714</v>
+      </c>
+      <c r="M229" t="n">
+        <v>0.254562998007102</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="s">
+        <v>31</v>
+      </c>
+      <c r="B230" t="s">
+        <v>24</v>
+      </c>
+      <c r="C230" t="s">
+        <v>20</v>
+      </c>
+      <c r="D230" t="s">
+        <v>16</v>
+      </c>
+      <c r="E230" t="n">
+        <v>15</v>
+      </c>
+      <c r="F230" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" t="n">
+        <v>0.0535714285714286</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" t="n">
+        <v>0.157171326650143</v>
+      </c>
+      <c r="K230"/>
+      <c r="L230"/>
+      <c r="M230"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="s">
+        <v>31</v>
+      </c>
+      <c r="B231" t="s">
+        <v>24</v>
+      </c>
+      <c r="C231" t="s">
+        <v>20</v>
+      </c>
+      <c r="D231" t="s">
+        <v>16</v>
+      </c>
+      <c r="E231" t="n">
+        <v>15</v>
+      </c>
+      <c r="F231" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G231" t="n">
+        <v>200</v>
+      </c>
+      <c r="H231" t="n">
+        <v>0.0535714285714286</v>
+      </c>
+      <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
+        <v>0.157171326650143</v>
+      </c>
+      <c r="K231" t="n">
+        <v>0.915422885572139</v>
+      </c>
+      <c r="L231" t="n">
+        <v>0.340803571428571</v>
+      </c>
+      <c r="M231" t="n">
+        <v>0.222839976899532</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="s">
+        <v>31</v>
+      </c>
+      <c r="B232" t="s">
+        <v>24</v>
+      </c>
+      <c r="C232" t="s">
+        <v>21</v>
+      </c>
+      <c r="D232" t="s">
+        <v>16</v>
+      </c>
+      <c r="E232" t="n">
+        <v>15</v>
+      </c>
+      <c r="F232" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" t="n">
+        <v>0</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>0</v>
+      </c>
+      <c r="K232"/>
+      <c r="L232"/>
+      <c r="M232"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="s">
+        <v>31</v>
+      </c>
+      <c r="B233" t="s">
+        <v>24</v>
+      </c>
+      <c r="C233" t="s">
+        <v>21</v>
+      </c>
+      <c r="D233" t="s">
+        <v>16</v>
+      </c>
+      <c r="E233" t="n">
+        <v>15</v>
+      </c>
+      <c r="F233" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G233" t="n">
+        <v>200</v>
+      </c>
+      <c r="H233" t="n">
+        <v>0</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" t="n">
+        <v>1</v>
+      </c>
+      <c r="L233" t="n">
+        <v>0.0351785714285714</v>
+      </c>
+      <c r="M233" t="n">
+        <v>0.140583463224855</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="s">
+        <v>31</v>
+      </c>
+      <c r="B234" t="s">
+        <v>24</v>
+      </c>
+      <c r="C234" t="s">
+        <v>22</v>
+      </c>
+      <c r="D234" t="s">
+        <v>16</v>
+      </c>
+      <c r="E234" t="n">
+        <v>15</v>
+      </c>
+      <c r="F234" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="n">
+        <v>0</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234"/>
+      <c r="L234"/>
+      <c r="M234"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="s">
+        <v>31</v>
+      </c>
+      <c r="B235" t="s">
+        <v>24</v>
+      </c>
+      <c r="C235" t="s">
+        <v>22</v>
+      </c>
+      <c r="D235" t="s">
+        <v>16</v>
+      </c>
+      <c r="E235" t="n">
+        <v>15</v>
+      </c>
+      <c r="F235" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G235" t="n">
+        <v>200</v>
+      </c>
+      <c r="H235" t="n">
+        <v>0</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K235" t="n">
+        <v>1</v>
+      </c>
+      <c r="L235" t="n">
+        <v>0.453392857142857</v>
+      </c>
+      <c r="M235" t="n">
+        <v>0.24831365149962</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="s">
+        <v>31</v>
+      </c>
+      <c r="B236" t="s">
+        <v>24</v>
+      </c>
+      <c r="C236" t="s">
+        <v>23</v>
+      </c>
+      <c r="D236" t="s">
+        <v>16</v>
+      </c>
+      <c r="E236" t="n">
+        <v>15</v>
+      </c>
+      <c r="F236" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" t="n">
+        <v>0.267857142857143</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>0.54344235441157</v>
+      </c>
+      <c r="K236"/>
+      <c r="L236"/>
+      <c r="M236"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="s">
+        <v>31</v>
+      </c>
+      <c r="B237" t="s">
+        <v>24</v>
+      </c>
+      <c r="C237" t="s">
+        <v>23</v>
+      </c>
+      <c r="D237" t="s">
+        <v>16</v>
+      </c>
+      <c r="E237" t="n">
+        <v>15</v>
+      </c>
+      <c r="F237" t="n">
+        <v>1903</v>
+      </c>
+      <c r="G237" t="n">
+        <v>200</v>
+      </c>
+      <c r="H237" t="n">
+        <v>0.267857142857143</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>0.54344235441157</v>
+      </c>
+      <c r="K237" t="n">
+        <v>0.577114427860697</v>
+      </c>
+      <c r="L237" t="n">
+        <v>0.341071428571429</v>
+      </c>
+      <c r="M237" t="n">
+        <v>0.254188833105631</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="s">
+        <v>31</v>
+      </c>
+      <c r="B238" t="s">
+        <v>25</v>
+      </c>
+      <c r="C238" t="s">
+        <v>15</v>
+      </c>
+      <c r="D238" t="s">
+        <v>16</v>
+      </c>
+      <c r="E238" t="n">
+        <v>15</v>
+      </c>
+      <c r="F238" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H238" t="n">
+        <v>0</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238"/>
+      <c r="L238"/>
+      <c r="M238"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="s">
+        <v>31</v>
+      </c>
+      <c r="B239" t="s">
+        <v>25</v>
+      </c>
+      <c r="C239" t="s">
+        <v>15</v>
+      </c>
+      <c r="D239" t="s">
+        <v>16</v>
+      </c>
+      <c r="E239" t="n">
+        <v>15</v>
+      </c>
+      <c r="F239" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G239" t="n">
+        <v>200</v>
+      </c>
+      <c r="H239" t="n">
+        <v>0</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" t="n">
+        <v>1</v>
+      </c>
+      <c r="L239" t="n">
+        <v>0.0909821428571428</v>
+      </c>
+      <c r="M239" t="n">
+        <v>0.202185886225931</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s">
+        <v>31</v>
+      </c>
+      <c r="B240" t="s">
+        <v>25</v>
+      </c>
+      <c r="C240" t="s">
+        <v>17</v>
+      </c>
+      <c r="D240" t="s">
+        <v>16</v>
+      </c>
+      <c r="E240" t="n">
+        <v>15</v>
+      </c>
+      <c r="F240" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G240" t="n">
+        <v>0</v>
+      </c>
+      <c r="H240" t="n">
+        <v>0</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>0</v>
+      </c>
+      <c r="K240"/>
+      <c r="L240"/>
+      <c r="M240"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="s">
+        <v>31</v>
+      </c>
+      <c r="B241" t="s">
+        <v>25</v>
+      </c>
+      <c r="C241" t="s">
+        <v>17</v>
+      </c>
+      <c r="D241" t="s">
+        <v>16</v>
+      </c>
+      <c r="E241" t="n">
+        <v>15</v>
+      </c>
+      <c r="F241" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G241" t="n">
+        <v>200</v>
+      </c>
+      <c r="H241" t="n">
+        <v>0</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K241" t="n">
+        <v>1</v>
+      </c>
+      <c r="L241" t="n">
+        <v>0.0804464285714286</v>
+      </c>
+      <c r="M241" t="n">
+        <v>0.192992673091462</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="s">
+        <v>31</v>
+      </c>
+      <c r="B242" t="s">
+        <v>25</v>
+      </c>
+      <c r="C242" t="s">
+        <v>18</v>
+      </c>
+      <c r="D242" t="s">
+        <v>16</v>
+      </c>
+      <c r="E242" t="n">
+        <v>15</v>
+      </c>
+      <c r="F242" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G242" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" t="n">
+        <v>0.0892857142857143</v>
+      </c>
+      <c r="I242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" t="n">
+        <v>0.270021615983094</v>
+      </c>
+      <c r="K242"/>
+      <c r="L242"/>
+      <c r="M242"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="s">
+        <v>31</v>
+      </c>
+      <c r="B243" t="s">
+        <v>25</v>
+      </c>
+      <c r="C243" t="s">
+        <v>18</v>
+      </c>
+      <c r="D243" t="s">
+        <v>16</v>
+      </c>
+      <c r="E243" t="n">
+        <v>15</v>
+      </c>
+      <c r="F243" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G243" t="n">
+        <v>200</v>
+      </c>
+      <c r="H243" t="n">
+        <v>0.0892857142857143</v>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="n">
+        <v>0.270021615983094</v>
+      </c>
+      <c r="K243" t="n">
+        <v>0.706467661691542</v>
+      </c>
+      <c r="L243" t="n">
+        <v>0.250892857142857</v>
+      </c>
+      <c r="M243" t="n">
+        <v>0.240431637520497</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="s">
+        <v>31</v>
+      </c>
+      <c r="B244" t="s">
+        <v>25</v>
+      </c>
+      <c r="C244" t="s">
+        <v>20</v>
+      </c>
+      <c r="D244" t="s">
+        <v>16</v>
+      </c>
+      <c r="E244" t="n">
+        <v>15</v>
+      </c>
+      <c r="F244" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G244" t="n">
+        <v>0</v>
+      </c>
+      <c r="H244" t="n">
+        <v>0.214285714285714</v>
+      </c>
+      <c r="I244" t="n">
+        <v>0</v>
+      </c>
+      <c r="J244" t="n">
+        <v>0.468397160033926</v>
+      </c>
+      <c r="K244"/>
+      <c r="L244"/>
+      <c r="M244"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="s">
+        <v>31</v>
+      </c>
+      <c r="B245" t="s">
+        <v>25</v>
+      </c>
+      <c r="C245" t="s">
+        <v>20</v>
+      </c>
+      <c r="D245" t="s">
+        <v>16</v>
+      </c>
+      <c r="E245" t="n">
+        <v>15</v>
+      </c>
+      <c r="F245" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G245" t="n">
+        <v>200</v>
+      </c>
+      <c r="H245" t="n">
+        <v>0.214285714285714</v>
+      </c>
+      <c r="I245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J245" t="n">
+        <v>0.468397160033926</v>
+      </c>
+      <c r="K245" t="n">
+        <v>0.592039800995025</v>
+      </c>
+      <c r="L245" t="n">
+        <v>0.288839285714286</v>
+      </c>
+      <c r="M245" t="n">
+        <v>0.212403777674221</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="s">
+        <v>31</v>
+      </c>
+      <c r="B246" t="s">
+        <v>25</v>
+      </c>
+      <c r="C246" t="s">
+        <v>21</v>
+      </c>
+      <c r="D246" t="s">
+        <v>16</v>
+      </c>
+      <c r="E246" t="n">
+        <v>15</v>
+      </c>
+      <c r="F246" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G246" t="n">
+        <v>0</v>
+      </c>
+      <c r="H246" t="n">
+        <v>0</v>
+      </c>
+      <c r="I246" t="n">
+        <v>0</v>
+      </c>
+      <c r="J246" t="n">
+        <v>0</v>
+      </c>
+      <c r="K246"/>
+      <c r="L246"/>
+      <c r="M246"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="s">
+        <v>31</v>
+      </c>
+      <c r="B247" t="s">
+        <v>25</v>
+      </c>
+      <c r="C247" t="s">
+        <v>21</v>
+      </c>
+      <c r="D247" t="s">
+        <v>16</v>
+      </c>
+      <c r="E247" t="n">
+        <v>15</v>
+      </c>
+      <c r="F247" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G247" t="n">
+        <v>200</v>
+      </c>
+      <c r="H247" t="n">
+        <v>0</v>
+      </c>
+      <c r="I247" t="n">
+        <v>0</v>
+      </c>
+      <c r="J247" t="n">
+        <v>0</v>
+      </c>
+      <c r="K247" t="n">
+        <v>1</v>
+      </c>
+      <c r="L247" t="n">
+        <v>0.0257142857142857</v>
+      </c>
+      <c r="M247" t="n">
+        <v>0.129373544827054</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="s">
+        <v>31</v>
+      </c>
+      <c r="B248" t="s">
+        <v>25</v>
+      </c>
+      <c r="C248" t="s">
+        <v>22</v>
+      </c>
+      <c r="D248" t="s">
+        <v>16</v>
+      </c>
+      <c r="E248" t="n">
+        <v>15</v>
+      </c>
+      <c r="F248" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="n">
+        <v>0.464285714285714</v>
+      </c>
+      <c r="I248" t="n">
+        <v>0.133749304679759</v>
+      </c>
+      <c r="J248" t="n">
+        <v>0.794822123891669</v>
+      </c>
+      <c r="K248"/>
+      <c r="L248"/>
+      <c r="M248"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="s">
+        <v>31</v>
+      </c>
+      <c r="B249" t="s">
+        <v>25</v>
+      </c>
+      <c r="C249" t="s">
+        <v>22</v>
+      </c>
+      <c r="D249" t="s">
+        <v>16</v>
+      </c>
+      <c r="E249" t="n">
+        <v>15</v>
+      </c>
+      <c r="F249" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G249" t="n">
+        <v>200</v>
+      </c>
+      <c r="H249" t="n">
+        <v>0.464285714285714</v>
+      </c>
+      <c r="I249" t="n">
+        <v>0.133749304679759</v>
+      </c>
+      <c r="J249" t="n">
+        <v>0.794822123891669</v>
+      </c>
+      <c r="K249" t="n">
+        <v>0.432835820895522</v>
+      </c>
+      <c r="L249" t="n">
+        <v>0.428035714285714</v>
+      </c>
+      <c r="M249" t="n">
+        <v>0.226789635715146</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="s">
+        <v>31</v>
+      </c>
+      <c r="B250" t="s">
+        <v>25</v>
+      </c>
+      <c r="C250" t="s">
+        <v>23</v>
+      </c>
+      <c r="D250" t="s">
+        <v>16</v>
+      </c>
+      <c r="E250" t="n">
+        <v>15</v>
+      </c>
+      <c r="F250" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G250" t="n">
+        <v>0</v>
+      </c>
+      <c r="H250" t="n">
+        <v>0.196428571428571</v>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="n">
+        <v>0.433067414378383</v>
+      </c>
+      <c r="K250"/>
+      <c r="L250"/>
+      <c r="M250"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="s">
+        <v>31</v>
+      </c>
+      <c r="B251" t="s">
+        <v>25</v>
+      </c>
+      <c r="C251" t="s">
+        <v>23</v>
+      </c>
+      <c r="D251" t="s">
+        <v>16</v>
+      </c>
+      <c r="E251" t="n">
+        <v>15</v>
+      </c>
+      <c r="F251" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G251" t="n">
+        <v>200</v>
+      </c>
+      <c r="H251" t="n">
+        <v>0.196428571428571</v>
+      </c>
+      <c r="I251" t="n">
+        <v>0</v>
+      </c>
+      <c r="J251" t="n">
+        <v>0.433067414378383</v>
+      </c>
+      <c r="K251" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="L251" t="n">
+        <v>0.351428571428571</v>
+      </c>
+      <c r="M251" t="n">
+        <v>0.259088713257252</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="s">
+        <v>31</v>
+      </c>
+      <c r="B252" t="s">
+        <v>26</v>
+      </c>
+      <c r="C252" t="s">
+        <v>15</v>
+      </c>
+      <c r="D252" t="s">
+        <v>16</v>
+      </c>
+      <c r="E252" t="n">
+        <v>15</v>
+      </c>
+      <c r="F252" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G252" t="n">
+        <v>0</v>
+      </c>
+      <c r="H252" t="n">
+        <v>0</v>
+      </c>
+      <c r="I252" t="n">
+        <v>0</v>
+      </c>
+      <c r="J252" t="n">
+        <v>0</v>
+      </c>
+      <c r="K252"/>
+      <c r="L252"/>
+      <c r="M252"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="s">
+        <v>31</v>
+      </c>
+      <c r="B253" t="s">
+        <v>26</v>
+      </c>
+      <c r="C253" t="s">
+        <v>15</v>
+      </c>
+      <c r="D253" t="s">
+        <v>16</v>
+      </c>
+      <c r="E253" t="n">
+        <v>15</v>
+      </c>
+      <c r="F253" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G253" t="n">
+        <v>200</v>
+      </c>
+      <c r="H253" t="n">
+        <v>0</v>
+      </c>
+      <c r="I253" t="n">
+        <v>0</v>
+      </c>
+      <c r="J253" t="n">
+        <v>0</v>
+      </c>
+      <c r="K253" t="n">
+        <v>1</v>
+      </c>
+      <c r="L253" t="n">
+        <v>0.0946428571428572</v>
+      </c>
+      <c r="M253" t="n">
+        <v>0.209361034739988</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="s">
+        <v>31</v>
+      </c>
+      <c r="B254" t="s">
+        <v>26</v>
+      </c>
+      <c r="C254" t="s">
+        <v>17</v>
+      </c>
+      <c r="D254" t="s">
+        <v>16</v>
+      </c>
+      <c r="E254" t="n">
+        <v>15</v>
+      </c>
+      <c r="F254" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="n">
+        <v>0.232142857142857</v>
+      </c>
+      <c r="I254" t="n">
+        <v>0</v>
+      </c>
+      <c r="J254" t="n">
+        <v>0.533218709048258</v>
+      </c>
+      <c r="K254"/>
+      <c r="L254"/>
+      <c r="M254"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="s">
+        <v>31</v>
+      </c>
+      <c r="B255" t="s">
+        <v>26</v>
+      </c>
+      <c r="C255" t="s">
+        <v>17</v>
+      </c>
+      <c r="D255" t="s">
+        <v>16</v>
+      </c>
+      <c r="E255" t="n">
+        <v>15</v>
+      </c>
+      <c r="F255" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G255" t="n">
+        <v>200</v>
+      </c>
+      <c r="H255" t="n">
+        <v>0.232142857142857</v>
+      </c>
+      <c r="I255" t="n">
+        <v>0</v>
+      </c>
+      <c r="J255" t="n">
+        <v>0.533218709048258</v>
+      </c>
+      <c r="K255" t="n">
+        <v>0.144278606965174</v>
+      </c>
+      <c r="L255" t="n">
+        <v>0.0985714285714286</v>
+      </c>
+      <c r="M255" t="n">
+        <v>0.211007467567123</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="s">
+        <v>31</v>
+      </c>
+      <c r="B256" t="s">
+        <v>26</v>
+      </c>
+      <c r="C256" t="s">
+        <v>18</v>
+      </c>
+      <c r="D256" t="s">
+        <v>16</v>
+      </c>
+      <c r="E256" t="n">
+        <v>15</v>
+      </c>
+      <c r="F256" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G256" t="n">
+        <v>0</v>
+      </c>
+      <c r="H256" t="n">
+        <v>0.232142857142857</v>
+      </c>
+      <c r="I256" t="n">
+        <v>0</v>
+      </c>
+      <c r="J256" t="n">
+        <v>0.539925007162735</v>
+      </c>
+      <c r="K256"/>
+      <c r="L256"/>
+      <c r="M256"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="s">
+        <v>31</v>
+      </c>
+      <c r="B257" t="s">
+        <v>26</v>
+      </c>
+      <c r="C257" t="s">
+        <v>18</v>
+      </c>
+      <c r="D257" t="s">
+        <v>16</v>
+      </c>
+      <c r="E257" t="n">
+        <v>15</v>
+      </c>
+      <c r="F257" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G257" t="n">
+        <v>200</v>
+      </c>
+      <c r="H257" t="n">
+        <v>0.232142857142857</v>
+      </c>
+      <c r="I257" t="n">
+        <v>0</v>
+      </c>
+      <c r="J257" t="n">
+        <v>0.539925007162735</v>
+      </c>
+      <c r="K257" t="n">
+        <v>0.447761194029851</v>
+      </c>
+      <c r="L257" t="n">
+        <v>0.239375</v>
+      </c>
+      <c r="M257" t="n">
+        <v>0.238130289879202</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="s">
+        <v>31</v>
+      </c>
+      <c r="B258" t="s">
+        <v>26</v>
+      </c>
+      <c r="C258" t="s">
+        <v>20</v>
+      </c>
+      <c r="D258" t="s">
+        <v>16</v>
+      </c>
+      <c r="E258" t="n">
+        <v>15</v>
+      </c>
+      <c r="F258" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" t="n">
+        <v>0.517857142857143</v>
+      </c>
+      <c r="I258" t="n">
+        <v>0.18311214263335</v>
+      </c>
+      <c r="J258" t="n">
+        <v>0.852602143080936</v>
+      </c>
+      <c r="K258"/>
+      <c r="L258"/>
+      <c r="M258"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="s">
+        <v>31</v>
+      </c>
+      <c r="B259" t="s">
+        <v>26</v>
+      </c>
+      <c r="C259" t="s">
+        <v>20</v>
+      </c>
+      <c r="D259" t="s">
+        <v>16</v>
+      </c>
+      <c r="E259" t="n">
+        <v>15</v>
+      </c>
+      <c r="F259" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G259" t="n">
+        <v>200</v>
+      </c>
+      <c r="H259" t="n">
+        <v>0.517857142857143</v>
+      </c>
+      <c r="I259" t="n">
+        <v>0.18311214263335</v>
+      </c>
+      <c r="J259" t="n">
+        <v>0.852602143080936</v>
+      </c>
+      <c r="K259" t="n">
+        <v>0.169154228855721</v>
+      </c>
+      <c r="L259" t="n">
+        <v>0.284285714285714</v>
+      </c>
+      <c r="M259" t="n">
+        <v>0.213163789487333</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="s">
+        <v>31</v>
+      </c>
+      <c r="B260" t="s">
+        <v>26</v>
+      </c>
+      <c r="C260" t="s">
+        <v>21</v>
+      </c>
+      <c r="D260" t="s">
+        <v>16</v>
+      </c>
+      <c r="E260" t="n">
+        <v>15</v>
+      </c>
+      <c r="F260" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="n">
+        <v>0</v>
+      </c>
+      <c r="I260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J260" t="n">
+        <v>0</v>
+      </c>
+      <c r="K260"/>
+      <c r="L260"/>
+      <c r="M260"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="s">
+        <v>31</v>
+      </c>
+      <c r="B261" t="s">
+        <v>26</v>
+      </c>
+      <c r="C261" t="s">
+        <v>21</v>
+      </c>
+      <c r="D261" t="s">
+        <v>16</v>
+      </c>
+      <c r="E261" t="n">
+        <v>15</v>
+      </c>
+      <c r="F261" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G261" t="n">
+        <v>200</v>
+      </c>
+      <c r="H261" t="n">
+        <v>0</v>
+      </c>
+      <c r="I261" t="n">
+        <v>0</v>
+      </c>
+      <c r="J261" t="n">
+        <v>0</v>
+      </c>
+      <c r="K261" t="n">
+        <v>1</v>
+      </c>
+      <c r="L261" t="n">
+        <v>0.01375</v>
+      </c>
+      <c r="M261" t="n">
+        <v>0.100931304575227</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="s">
+        <v>31</v>
+      </c>
+      <c r="B262" t="s">
+        <v>26</v>
+      </c>
+      <c r="C262" t="s">
+        <v>22</v>
+      </c>
+      <c r="D262" t="s">
+        <v>16</v>
+      </c>
+      <c r="E262" t="n">
+        <v>15</v>
+      </c>
+      <c r="F262" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G262" t="n">
+        <v>0</v>
+      </c>
+      <c r="H262" t="n">
+        <v>0.482142857142857</v>
+      </c>
+      <c r="I262" t="n">
+        <v>0.161095801432675</v>
+      </c>
+      <c r="J262" t="n">
+        <v>0.803189912853039</v>
+      </c>
+      <c r="K262"/>
+      <c r="L262"/>
+      <c r="M262"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="s">
+        <v>31</v>
+      </c>
+      <c r="B263" t="s">
+        <v>26</v>
+      </c>
+      <c r="C263" t="s">
+        <v>22</v>
+      </c>
+      <c r="D263" t="s">
+        <v>16</v>
+      </c>
+      <c r="E263" t="n">
+        <v>15</v>
+      </c>
+      <c r="F263" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G263" t="n">
+        <v>200</v>
+      </c>
+      <c r="H263" t="n">
+        <v>0.482142857142857</v>
+      </c>
+      <c r="I263" t="n">
+        <v>0.161095801432675</v>
+      </c>
+      <c r="J263" t="n">
+        <v>0.803189912853039</v>
+      </c>
+      <c r="K263" t="n">
+        <v>0.36318407960199</v>
+      </c>
+      <c r="L263" t="n">
+        <v>0.398839285714286</v>
+      </c>
+      <c r="M263" t="n">
+        <v>0.237147024214376</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="s">
+        <v>31</v>
+      </c>
+      <c r="B264" t="s">
+        <v>26</v>
+      </c>
+      <c r="C264" t="s">
+        <v>23</v>
+      </c>
+      <c r="D264" t="s">
+        <v>16</v>
+      </c>
+      <c r="E264" t="n">
+        <v>15</v>
+      </c>
+      <c r="F264" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G264" t="n">
+        <v>0</v>
+      </c>
+      <c r="H264" t="n">
+        <v>0</v>
+      </c>
+      <c r="I264" t="n">
+        <v>0</v>
+      </c>
+      <c r="J264" t="n">
+        <v>0</v>
+      </c>
+      <c r="K264"/>
+      <c r="L264"/>
+      <c r="M264"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="s">
+        <v>31</v>
+      </c>
+      <c r="B265" t="s">
+        <v>26</v>
+      </c>
+      <c r="C265" t="s">
+        <v>23</v>
+      </c>
+      <c r="D265" t="s">
+        <v>16</v>
+      </c>
+      <c r="E265" t="n">
+        <v>15</v>
+      </c>
+      <c r="F265" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G265" t="n">
+        <v>200</v>
+      </c>
+      <c r="H265" t="n">
+        <v>0</v>
+      </c>
+      <c r="I265" t="n">
+        <v>0</v>
+      </c>
+      <c r="J265" t="n">
+        <v>0</v>
+      </c>
+      <c r="K265" t="n">
+        <v>1</v>
+      </c>
+      <c r="L265" t="n">
+        <v>0.333303571428571</v>
+      </c>
+      <c r="M265" t="n">
+        <v>0.253217916197242</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="s">
+        <v>31</v>
+      </c>
+      <c r="B266" t="s">
+        <v>27</v>
+      </c>
+      <c r="C266" t="s">
+        <v>15</v>
+      </c>
+      <c r="D266" t="s">
+        <v>16</v>
+      </c>
+      <c r="E266" t="n">
+        <v>14</v>
+      </c>
+      <c r="F266" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H266" t="n">
+        <v>0</v>
+      </c>
+      <c r="I266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J266" t="n">
+        <v>0</v>
+      </c>
+      <c r="K266"/>
+      <c r="L266"/>
+      <c r="M266"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="s">
+        <v>31</v>
+      </c>
+      <c r="B267" t="s">
+        <v>27</v>
+      </c>
+      <c r="C267" t="s">
+        <v>15</v>
+      </c>
+      <c r="D267" t="s">
+        <v>16</v>
+      </c>
+      <c r="E267" t="n">
+        <v>14</v>
+      </c>
+      <c r="F267" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G267" t="n">
+        <v>200</v>
+      </c>
+      <c r="H267" t="n">
+        <v>0</v>
+      </c>
+      <c r="I267" t="n">
+        <v>0</v>
+      </c>
+      <c r="J267" t="n">
+        <v>0</v>
+      </c>
+      <c r="K267" t="n">
+        <v>1</v>
+      </c>
+      <c r="L267" t="n">
+        <v>0.0908333333333334</v>
+      </c>
+      <c r="M267" t="n">
+        <v>0.204391519774347</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="s">
+        <v>31</v>
+      </c>
+      <c r="B268" t="s">
+        <v>27</v>
+      </c>
+      <c r="C268" t="s">
+        <v>17</v>
+      </c>
+      <c r="D268" t="s">
+        <v>16</v>
+      </c>
+      <c r="E268" t="n">
+        <v>14</v>
+      </c>
+      <c r="F268" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="n">
+        <v>0</v>
+      </c>
+      <c r="I268" t="n">
+        <v>0</v>
+      </c>
+      <c r="J268" t="n">
+        <v>0</v>
+      </c>
+      <c r="K268"/>
+      <c r="L268"/>
+      <c r="M268"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="s">
+        <v>31</v>
+      </c>
+      <c r="B269" t="s">
+        <v>27</v>
+      </c>
+      <c r="C269" t="s">
+        <v>17</v>
+      </c>
+      <c r="D269" t="s">
+        <v>16</v>
+      </c>
+      <c r="E269" t="n">
+        <v>14</v>
+      </c>
+      <c r="F269" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G269" t="n">
+        <v>200</v>
+      </c>
+      <c r="H269" t="n">
+        <v>0</v>
+      </c>
+      <c r="I269" t="n">
+        <v>0</v>
+      </c>
+      <c r="J269" t="n">
+        <v>0</v>
+      </c>
+      <c r="K269" t="n">
+        <v>1</v>
+      </c>
+      <c r="L269" t="n">
+        <v>0.112291666666667</v>
+      </c>
+      <c r="M269" t="n">
+        <v>0.231348020106149</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="s">
+        <v>31</v>
+      </c>
+      <c r="B270" t="s">
+        <v>27</v>
+      </c>
+      <c r="C270" t="s">
+        <v>18</v>
+      </c>
+      <c r="D270" t="s">
+        <v>16</v>
+      </c>
+      <c r="E270" t="n">
+        <v>14</v>
+      </c>
+      <c r="F270" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G270" t="n">
+        <v>0</v>
+      </c>
+      <c r="H270" t="n">
+        <v>0</v>
+      </c>
+      <c r="I270" t="n">
+        <v>0</v>
+      </c>
+      <c r="J270" t="n">
+        <v>0</v>
+      </c>
+      <c r="K270"/>
+      <c r="L270"/>
+      <c r="M270"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="s">
+        <v>31</v>
+      </c>
+      <c r="B271" t="s">
+        <v>27</v>
+      </c>
+      <c r="C271" t="s">
+        <v>18</v>
+      </c>
+      <c r="D271" t="s">
+        <v>16</v>
+      </c>
+      <c r="E271" t="n">
+        <v>14</v>
+      </c>
+      <c r="F271" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G271" t="n">
+        <v>200</v>
+      </c>
+      <c r="H271" t="n">
+        <v>0</v>
+      </c>
+      <c r="I271" t="n">
+        <v>0</v>
+      </c>
+      <c r="J271" t="n">
+        <v>0</v>
+      </c>
+      <c r="K271" t="n">
+        <v>1</v>
+      </c>
+      <c r="L271" t="n">
+        <v>0.174739583333333</v>
+      </c>
+      <c r="M271" t="n">
+        <v>0.254629879127735</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="s">
+        <v>31</v>
+      </c>
+      <c r="B272" t="s">
+        <v>27</v>
+      </c>
+      <c r="C272" t="s">
+        <v>20</v>
+      </c>
+      <c r="D272" t="s">
+        <v>16</v>
+      </c>
+      <c r="E272" t="n">
+        <v>14</v>
+      </c>
+      <c r="F272" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="n">
+        <v>0</v>
+      </c>
+      <c r="I272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J272" t="n">
+        <v>0</v>
+      </c>
+      <c r="K272"/>
+      <c r="L272"/>
+      <c r="M272"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="s">
+        <v>31</v>
+      </c>
+      <c r="B273" t="s">
+        <v>27</v>
+      </c>
+      <c r="C273" t="s">
+        <v>20</v>
+      </c>
+      <c r="D273" t="s">
+        <v>16</v>
+      </c>
+      <c r="E273" t="n">
+        <v>14</v>
+      </c>
+      <c r="F273" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G273" t="n">
+        <v>200</v>
+      </c>
+      <c r="H273" t="n">
+        <v>0</v>
+      </c>
+      <c r="I273" t="n">
+        <v>0</v>
+      </c>
+      <c r="J273" t="n">
+        <v>0</v>
+      </c>
+      <c r="K273" t="n">
+        <v>1</v>
+      </c>
+      <c r="L273" t="n">
+        <v>0.271041666666667</v>
+      </c>
+      <c r="M273" t="n">
+        <v>0.198050129116888</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="s">
+        <v>31</v>
+      </c>
+      <c r="B274" t="s">
+        <v>27</v>
+      </c>
+      <c r="C274" t="s">
+        <v>21</v>
+      </c>
+      <c r="D274" t="s">
+        <v>16</v>
+      </c>
+      <c r="E274" t="n">
+        <v>14</v>
+      </c>
+      <c r="F274" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="n">
+        <v>0</v>
+      </c>
+      <c r="I274" t="n">
+        <v>0</v>
+      </c>
+      <c r="J274" t="n">
+        <v>0</v>
+      </c>
+      <c r="K274"/>
+      <c r="L274"/>
+      <c r="M274"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="s">
+        <v>31</v>
+      </c>
+      <c r="B275" t="s">
+        <v>27</v>
+      </c>
+      <c r="C275" t="s">
+        <v>21</v>
+      </c>
+      <c r="D275" t="s">
+        <v>16</v>
+      </c>
+      <c r="E275" t="n">
+        <v>14</v>
+      </c>
+      <c r="F275" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G275" t="n">
+        <v>200</v>
+      </c>
+      <c r="H275" t="n">
+        <v>0</v>
+      </c>
+      <c r="I275" t="n">
+        <v>0</v>
+      </c>
+      <c r="J275" t="n">
+        <v>0</v>
+      </c>
+      <c r="K275" t="n">
+        <v>1</v>
+      </c>
+      <c r="L275" t="n">
+        <v>0.0204166666666667</v>
+      </c>
+      <c r="M275" t="n">
+        <v>0.0923928144435703</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="s">
+        <v>31</v>
+      </c>
+      <c r="B276" t="s">
+        <v>27</v>
+      </c>
+      <c r="C276" t="s">
+        <v>22</v>
+      </c>
+      <c r="D276" t="s">
+        <v>16</v>
+      </c>
+      <c r="E276" t="n">
+        <v>14</v>
+      </c>
+      <c r="F276" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G276" t="n">
+        <v>0</v>
+      </c>
+      <c r="H276" t="n">
+        <v>0.229166666666667</v>
+      </c>
+      <c r="I276" t="n">
+        <v>0</v>
+      </c>
+      <c r="J276" t="n">
+        <v>0.526672637512813</v>
+      </c>
+      <c r="K276"/>
+      <c r="L276"/>
+      <c r="M276"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="s">
+        <v>31</v>
+      </c>
+      <c r="B277" t="s">
+        <v>27</v>
+      </c>
+      <c r="C277" t="s">
+        <v>22</v>
+      </c>
+      <c r="D277" t="s">
+        <v>16</v>
+      </c>
+      <c r="E277" t="n">
+        <v>14</v>
+      </c>
+      <c r="F277" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G277" t="n">
+        <v>200</v>
+      </c>
+      <c r="H277" t="n">
+        <v>0.229166666666667</v>
+      </c>
+      <c r="I277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J277" t="n">
+        <v>0.526672637512813</v>
+      </c>
+      <c r="K277" t="n">
+        <v>0.736318407960199</v>
+      </c>
+      <c r="L277" t="n">
+        <v>0.421770833333333</v>
+      </c>
+      <c r="M277" t="n">
+        <v>0.259759409277899</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="s">
+        <v>31</v>
+      </c>
+      <c r="B278" t="s">
+        <v>27</v>
+      </c>
+      <c r="C278" t="s">
+        <v>23</v>
+      </c>
+      <c r="D278" t="s">
+        <v>16</v>
+      </c>
+      <c r="E278" t="n">
+        <v>14</v>
+      </c>
+      <c r="F278" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="I278" t="n">
+        <v>0.0359268895893308</v>
+      </c>
+      <c r="J278" t="n">
+        <v>0.672406443744003</v>
+      </c>
+      <c r="K278"/>
+      <c r="L278"/>
+      <c r="M278"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="s">
+        <v>31</v>
+      </c>
+      <c r="B279" t="s">
+        <v>27</v>
+      </c>
+      <c r="C279" t="s">
+        <v>23</v>
+      </c>
+      <c r="D279" t="s">
+        <v>16</v>
+      </c>
+      <c r="E279" t="n">
+        <v>14</v>
+      </c>
+      <c r="F279" t="n">
+        <v>1905</v>
+      </c>
+      <c r="G279" t="n">
+        <v>200</v>
+      </c>
+      <c r="H279" t="n">
+        <v>0.354166666666667</v>
+      </c>
+      <c r="I279" t="n">
+        <v>0.0359268895893308</v>
+      </c>
+      <c r="J279" t="n">
+        <v>0.672406443744003</v>
+      </c>
+      <c r="K279" t="n">
+        <v>0.462686567164179</v>
+      </c>
+      <c r="L279" t="n">
+        <v>0.338645833333333</v>
+      </c>
+      <c r="M279" t="n">
+        <v>0.270990302888299</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="s">
+        <v>31</v>
+      </c>
+      <c r="B280" t="s">
+        <v>28</v>
+      </c>
+      <c r="C280" t="s">
+        <v>15</v>
+      </c>
+      <c r="D280" t="s">
+        <v>16</v>
+      </c>
+      <c r="E280" t="n">
+        <v>14</v>
+      </c>
+      <c r="F280" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G280" t="n">
+        <v>0</v>
+      </c>
+      <c r="H280" t="n">
+        <v>0</v>
+      </c>
+      <c r="I280" t="n">
+        <v>0</v>
+      </c>
+      <c r="J280" t="n">
+        <v>0</v>
+      </c>
+      <c r="K280"/>
+      <c r="L280"/>
+      <c r="M280"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="s">
+        <v>31</v>
+      </c>
+      <c r="B281" t="s">
+        <v>28</v>
+      </c>
+      <c r="C281" t="s">
+        <v>15</v>
+      </c>
+      <c r="D281" t="s">
+        <v>16</v>
+      </c>
+      <c r="E281" t="n">
+        <v>14</v>
+      </c>
+      <c r="F281" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G281" t="n">
+        <v>200</v>
+      </c>
+      <c r="H281" t="n">
+        <v>0</v>
+      </c>
+      <c r="I281" t="n">
+        <v>0</v>
+      </c>
+      <c r="J281" t="n">
+        <v>0</v>
+      </c>
+      <c r="K281" t="n">
+        <v>1</v>
+      </c>
+      <c r="L281" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="M281" t="n">
+        <v>0.160167460174393</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="s">
+        <v>31</v>
+      </c>
+      <c r="B282" t="s">
+        <v>28</v>
+      </c>
+      <c r="C282" t="s">
+        <v>17</v>
+      </c>
+      <c r="D282" t="s">
+        <v>16</v>
+      </c>
+      <c r="E282" t="n">
+        <v>14</v>
+      </c>
+      <c r="F282" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G282" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" t="n">
+        <v>0</v>
+      </c>
+      <c r="I282" t="n">
+        <v>0</v>
+      </c>
+      <c r="J282" t="n">
+        <v>0</v>
+      </c>
+      <c r="K282"/>
+      <c r="L282"/>
+      <c r="M282"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="s">
+        <v>31</v>
+      </c>
+      <c r="B283" t="s">
+        <v>28</v>
+      </c>
+      <c r="C283" t="s">
+        <v>17</v>
+      </c>
+      <c r="D283" t="s">
+        <v>16</v>
+      </c>
+      <c r="E283" t="n">
+        <v>14</v>
+      </c>
+      <c r="F283" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G283" t="n">
+        <v>200</v>
+      </c>
+      <c r="H283" t="n">
+        <v>0</v>
+      </c>
+      <c r="I283" t="n">
+        <v>0</v>
+      </c>
+      <c r="J283" t="n">
+        <v>0</v>
+      </c>
+      <c r="K283" t="n">
+        <v>1</v>
+      </c>
+      <c r="L283" t="n">
+        <v>0.0710416666666667</v>
+      </c>
+      <c r="M283" t="n">
+        <v>0.189256268487786</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="s">
+        <v>31</v>
+      </c>
+      <c r="B284" t="s">
+        <v>28</v>
+      </c>
+      <c r="C284" t="s">
+        <v>18</v>
+      </c>
+      <c r="D284" t="s">
+        <v>16</v>
+      </c>
+      <c r="E284" t="n">
+        <v>14</v>
+      </c>
+      <c r="F284" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G284" t="n">
+        <v>0</v>
+      </c>
+      <c r="H284" t="n">
+        <v>0</v>
+      </c>
+      <c r="I284" t="n">
+        <v>0</v>
+      </c>
+      <c r="J284" t="n">
+        <v>0</v>
+      </c>
+      <c r="K284"/>
+      <c r="L284"/>
+      <c r="M284"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="s">
+        <v>31</v>
+      </c>
+      <c r="B285" t="s">
+        <v>28</v>
+      </c>
+      <c r="C285" t="s">
+        <v>18</v>
+      </c>
+      <c r="D285" t="s">
+        <v>16</v>
+      </c>
+      <c r="E285" t="n">
+        <v>14</v>
+      </c>
+      <c r="F285" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G285" t="n">
+        <v>200</v>
+      </c>
+      <c r="H285" t="n">
+        <v>0</v>
+      </c>
+      <c r="I285" t="n">
+        <v>0</v>
+      </c>
+      <c r="J285" t="n">
+        <v>0</v>
+      </c>
+      <c r="K285" t="n">
+        <v>1</v>
+      </c>
+      <c r="L285" t="n">
+        <v>0.185833333333333</v>
+      </c>
+      <c r="M285" t="n">
+        <v>0.251568571628405</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="s">
+        <v>31</v>
+      </c>
+      <c r="B286" t="s">
+        <v>28</v>
+      </c>
+      <c r="C286" t="s">
+        <v>20</v>
+      </c>
+      <c r="D286" t="s">
+        <v>16</v>
+      </c>
+      <c r="E286" t="n">
+        <v>14</v>
+      </c>
+      <c r="F286" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I286" t="n">
+        <v>0</v>
+      </c>
+      <c r="J286" t="n">
+        <v>0.618818397935346</v>
+      </c>
+      <c r="K286"/>
+      <c r="L286"/>
+      <c r="M286"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="s">
+        <v>31</v>
+      </c>
+      <c r="B287" t="s">
+        <v>28</v>
+      </c>
+      <c r="C287" t="s">
+        <v>20</v>
+      </c>
+      <c r="D287" t="s">
+        <v>16</v>
+      </c>
+      <c r="E287" t="n">
+        <v>14</v>
+      </c>
+      <c r="F287" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G287" t="n">
+        <v>200</v>
+      </c>
+      <c r="H287" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I287" t="n">
+        <v>0</v>
+      </c>
+      <c r="J287" t="n">
+        <v>0.618818397935346</v>
+      </c>
+      <c r="K287" t="n">
+        <v>0.447761194029851</v>
+      </c>
+      <c r="L287" t="n">
+        <v>0.264583333333333</v>
+      </c>
+      <c r="M287" t="n">
+        <v>0.212910358532692</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="s">
+        <v>31</v>
+      </c>
+      <c r="B288" t="s">
+        <v>28</v>
+      </c>
+      <c r="C288" t="s">
+        <v>21</v>
+      </c>
+      <c r="D288" t="s">
+        <v>16</v>
+      </c>
+      <c r="E288" t="n">
+        <v>14</v>
+      </c>
+      <c r="F288" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0</v>
+      </c>
+      <c r="H288" t="n">
+        <v>0</v>
+      </c>
+      <c r="I288" t="n">
+        <v>0</v>
+      </c>
+      <c r="J288" t="n">
+        <v>0</v>
+      </c>
+      <c r="K288"/>
+      <c r="L288"/>
+      <c r="M288"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="s">
+        <v>31</v>
+      </c>
+      <c r="B289" t="s">
+        <v>28</v>
+      </c>
+      <c r="C289" t="s">
+        <v>21</v>
+      </c>
+      <c r="D289" t="s">
+        <v>16</v>
+      </c>
+      <c r="E289" t="n">
+        <v>14</v>
+      </c>
+      <c r="F289" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G289" t="n">
+        <v>200</v>
+      </c>
+      <c r="H289" t="n">
+        <v>0</v>
+      </c>
+      <c r="I289" t="n">
+        <v>0</v>
+      </c>
+      <c r="J289" t="n">
+        <v>0</v>
+      </c>
+      <c r="K289" t="n">
+        <v>1</v>
+      </c>
+      <c r="L289" t="n">
+        <v>0.0157291666666667</v>
+      </c>
+      <c r="M289" t="n">
+        <v>0.115919807854461</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="s">
+        <v>31</v>
+      </c>
+      <c r="B290" t="s">
+        <v>28</v>
+      </c>
+      <c r="C290" t="s">
+        <v>22</v>
+      </c>
+      <c r="D290" t="s">
+        <v>16</v>
+      </c>
+      <c r="E290" t="n">
+        <v>14</v>
+      </c>
+      <c r="F290" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="n">
+        <v>0.229166666666667</v>
+      </c>
+      <c r="I290" t="n">
+        <v>0</v>
+      </c>
+      <c r="J290" t="n">
+        <v>0.559741310164942</v>
+      </c>
+      <c r="K290"/>
+      <c r="L290"/>
+      <c r="M290"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="s">
+        <v>31</v>
+      </c>
+      <c r="B291" t="s">
+        <v>28</v>
+      </c>
+      <c r="C291" t="s">
+        <v>22</v>
+      </c>
+      <c r="D291" t="s">
+        <v>16</v>
+      </c>
+      <c r="E291" t="n">
+        <v>14</v>
+      </c>
+      <c r="F291" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G291" t="n">
+        <v>200</v>
+      </c>
+      <c r="H291" t="n">
+        <v>0.229166666666667</v>
+      </c>
+      <c r="I291" t="n">
+        <v>0</v>
+      </c>
+      <c r="J291" t="n">
+        <v>0.559741310164942</v>
+      </c>
+      <c r="K291" t="n">
+        <v>0.741293532338308</v>
+      </c>
+      <c r="L291" t="n">
+        <v>0.421041666666667</v>
+      </c>
+      <c r="M291" t="n">
+        <v>0.245533363958673</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="s">
+        <v>31</v>
+      </c>
+      <c r="B292" t="s">
+        <v>28</v>
+      </c>
+      <c r="C292" t="s">
+        <v>23</v>
+      </c>
+      <c r="D292" t="s">
+        <v>16</v>
+      </c>
+      <c r="E292" t="n">
+        <v>14</v>
+      </c>
+      <c r="F292" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0</v>
+      </c>
+      <c r="H292" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="I292" t="n">
+        <v>0.217333835399937</v>
+      </c>
+      <c r="J292" t="n">
+        <v>0.94933283126673</v>
+      </c>
+      <c r="K292"/>
+      <c r="L292"/>
+      <c r="M292"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="s">
+        <v>31</v>
+      </c>
+      <c r="B293" t="s">
+        <v>28</v>
+      </c>
+      <c r="C293" t="s">
+        <v>23</v>
+      </c>
+      <c r="D293" t="s">
+        <v>16</v>
+      </c>
+      <c r="E293" t="n">
+        <v>14</v>
+      </c>
+      <c r="F293" t="n">
+        <v>1904</v>
+      </c>
+      <c r="G293" t="n">
+        <v>200</v>
+      </c>
+      <c r="H293" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="I293" t="n">
+        <v>0.217333835399937</v>
+      </c>
+      <c r="J293" t="n">
+        <v>0.94933283126673</v>
+      </c>
+      <c r="K293" t="n">
+        <v>0.174129353233831</v>
+      </c>
+      <c r="L293" t="n">
+        <v>0.313645833333333</v>
+      </c>
+      <c r="M293" t="n">
+        <v>0.262853527294459</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="s">
+        <v>31</v>
+      </c>
+      <c r="B294" t="s">
+        <v>29</v>
+      </c>
+      <c r="C294" t="s">
+        <v>15</v>
+      </c>
+      <c r="D294" t="s">
+        <v>16</v>
+      </c>
+      <c r="E294" t="n">
+        <v>14</v>
+      </c>
+      <c r="F294" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0</v>
+      </c>
+      <c r="H294" t="n">
+        <v>0</v>
+      </c>
+      <c r="I294" t="n">
+        <v>0</v>
+      </c>
+      <c r="J294" t="n">
+        <v>0</v>
+      </c>
+      <c r="K294"/>
+      <c r="L294"/>
+      <c r="M294"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="s">
+        <v>31</v>
+      </c>
+      <c r="B295" t="s">
+        <v>29</v>
+      </c>
+      <c r="C295" t="s">
+        <v>15</v>
+      </c>
+      <c r="D295" t="s">
+        <v>16</v>
+      </c>
+      <c r="E295" t="n">
+        <v>14</v>
+      </c>
+      <c r="F295" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G295" t="n">
+        <v>200</v>
+      </c>
+      <c r="H295" t="n">
+        <v>0</v>
+      </c>
+      <c r="I295" t="n">
+        <v>0</v>
+      </c>
+      <c r="J295" t="n">
+        <v>0</v>
+      </c>
+      <c r="K295" t="n">
+        <v>1</v>
+      </c>
+      <c r="L295" t="n">
+        <v>0.04625</v>
+      </c>
+      <c r="M295" t="n">
+        <v>0.137324452681594</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="s">
+        <v>31</v>
+      </c>
+      <c r="B296" t="s">
+        <v>29</v>
+      </c>
+      <c r="C296" t="s">
+        <v>17</v>
+      </c>
+      <c r="D296" t="s">
+        <v>16</v>
+      </c>
+      <c r="E296" t="n">
+        <v>14</v>
+      </c>
+      <c r="F296" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="n">
+        <v>0</v>
+      </c>
+      <c r="I296" t="n">
+        <v>0</v>
+      </c>
+      <c r="J296" t="n">
+        <v>0</v>
+      </c>
+      <c r="K296"/>
+      <c r="L296"/>
+      <c r="M296"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="s">
+        <v>31</v>
+      </c>
+      <c r="B297" t="s">
+        <v>29</v>
+      </c>
+      <c r="C297" t="s">
+        <v>17</v>
+      </c>
+      <c r="D297" t="s">
+        <v>16</v>
+      </c>
+      <c r="E297" t="n">
+        <v>14</v>
+      </c>
+      <c r="F297" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G297" t="n">
+        <v>200</v>
+      </c>
+      <c r="H297" t="n">
+        <v>0</v>
+      </c>
+      <c r="I297" t="n">
+        <v>0</v>
+      </c>
+      <c r="J297" t="n">
+        <v>0</v>
+      </c>
+      <c r="K297" t="n">
+        <v>1</v>
+      </c>
+      <c r="L297" t="n">
+        <v>0.0666666666666667</v>
+      </c>
+      <c r="M297" t="n">
+        <v>0.16368245428363</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="s">
+        <v>31</v>
+      </c>
+      <c r="B298" t="s">
+        <v>29</v>
+      </c>
+      <c r="C298" t="s">
+        <v>18</v>
+      </c>
+      <c r="D298" t="s">
+        <v>16</v>
+      </c>
+      <c r="E298" t="n">
+        <v>14</v>
+      </c>
+      <c r="F298" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0</v>
+      </c>
+      <c r="H298" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
+        <v>0.369995498067507</v>
+      </c>
+      <c r="K298"/>
+      <c r="L298"/>
+      <c r="M298"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="s">
+        <v>31</v>
+      </c>
+      <c r="B299" t="s">
+        <v>29</v>
+      </c>
+      <c r="C299" t="s">
+        <v>18</v>
+      </c>
+      <c r="D299" t="s">
+        <v>16</v>
+      </c>
+      <c r="E299" t="n">
+        <v>14</v>
+      </c>
+      <c r="F299" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G299" t="n">
+        <v>200</v>
+      </c>
+      <c r="H299" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="I299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J299" t="n">
+        <v>0.369995498067507</v>
+      </c>
+      <c r="K299" t="n">
+        <v>0.417910447761194</v>
+      </c>
+      <c r="L299" t="n">
+        <v>0.160833333333333</v>
+      </c>
+      <c r="M299" t="n">
+        <v>0.236062035084323</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="s">
+        <v>31</v>
+      </c>
+      <c r="B300" t="s">
+        <v>29</v>
+      </c>
+      <c r="C300" t="s">
+        <v>20</v>
+      </c>
+      <c r="D300" t="s">
+        <v>16</v>
+      </c>
+      <c r="E300" t="n">
+        <v>14</v>
+      </c>
+      <c r="F300" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0</v>
+      </c>
+      <c r="H300" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I300" t="n">
+        <v>0</v>
+      </c>
+      <c r="J300" t="n">
+        <v>0.55119252785563</v>
+      </c>
+      <c r="K300"/>
+      <c r="L300"/>
+      <c r="M300"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="s">
+        <v>31</v>
+      </c>
+      <c r="B301" t="s">
+        <v>29</v>
+      </c>
+      <c r="C301" t="s">
+        <v>20</v>
+      </c>
+      <c r="D301" t="s">
+        <v>16</v>
+      </c>
+      <c r="E301" t="n">
+        <v>14</v>
+      </c>
+      <c r="F301" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G301" t="n">
+        <v>200</v>
+      </c>
+      <c r="H301" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I301" t="n">
+        <v>0</v>
+      </c>
+      <c r="J301" t="n">
+        <v>0.55119252785563</v>
+      </c>
+      <c r="K301" t="n">
+        <v>0.378109452736318</v>
+      </c>
+      <c r="L301" t="n">
+        <v>0.216770833333333</v>
+      </c>
+      <c r="M301" t="n">
+        <v>0.19408002749784</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="s">
+        <v>31</v>
+      </c>
+      <c r="B302" t="s">
+        <v>29</v>
+      </c>
+      <c r="C302" t="s">
+        <v>21</v>
+      </c>
+      <c r="D302" t="s">
+        <v>16</v>
+      </c>
+      <c r="E302" t="n">
+        <v>14</v>
+      </c>
+      <c r="F302" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" t="n">
+        <v>0</v>
+      </c>
+      <c r="I302" t="n">
+        <v>0</v>
+      </c>
+      <c r="J302" t="n">
+        <v>0</v>
+      </c>
+      <c r="K302"/>
+      <c r="L302"/>
+      <c r="M302"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="s">
+        <v>31</v>
+      </c>
+      <c r="B303" t="s">
+        <v>29</v>
+      </c>
+      <c r="C303" t="s">
+        <v>21</v>
+      </c>
+      <c r="D303" t="s">
+        <v>16</v>
+      </c>
+      <c r="E303" t="n">
+        <v>14</v>
+      </c>
+      <c r="F303" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G303" t="n">
+        <v>200</v>
+      </c>
+      <c r="H303" t="n">
+        <v>0</v>
+      </c>
+      <c r="I303" t="n">
+        <v>0</v>
+      </c>
+      <c r="J303" t="n">
+        <v>0</v>
+      </c>
+      <c r="K303" t="n">
+        <v>1</v>
+      </c>
+      <c r="L303" t="n">
+        <v>0.0078125</v>
+      </c>
+      <c r="M303" t="n">
+        <v>0.0735291487559752</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="s">
+        <v>31</v>
+      </c>
+      <c r="B304" t="s">
+        <v>29</v>
+      </c>
+      <c r="C304" t="s">
+        <v>22</v>
+      </c>
+      <c r="D304" t="s">
+        <v>16</v>
+      </c>
+      <c r="E304" t="n">
+        <v>14</v>
+      </c>
+      <c r="F304" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0</v>
+      </c>
+      <c r="H304" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I304" t="n">
+        <v>0</v>
+      </c>
+      <c r="J304" t="n">
+        <v>0.551871364671475</v>
+      </c>
+      <c r="K304"/>
+      <c r="L304"/>
+      <c r="M304"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="s">
+        <v>31</v>
+      </c>
+      <c r="B305" t="s">
+        <v>29</v>
+      </c>
+      <c r="C305" t="s">
+        <v>22</v>
+      </c>
+      <c r="D305" t="s">
+        <v>16</v>
+      </c>
+      <c r="E305" t="n">
+        <v>14</v>
+      </c>
+      <c r="F305" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G305" t="n">
+        <v>200</v>
+      </c>
+      <c r="H305" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I305" t="n">
+        <v>0</v>
+      </c>
+      <c r="J305" t="n">
+        <v>0.551871364671475</v>
+      </c>
+      <c r="K305" t="n">
+        <v>0.641791044776119</v>
+      </c>
+      <c r="L305" t="n">
+        <v>0.4065625</v>
+      </c>
+      <c r="M305" t="n">
+        <v>0.256731483928585</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="s">
+        <v>31</v>
+      </c>
+      <c r="B306" t="s">
+        <v>29</v>
+      </c>
+      <c r="C306" t="s">
+        <v>23</v>
+      </c>
+      <c r="D306" t="s">
+        <v>16</v>
+      </c>
+      <c r="E306" t="n">
+        <v>14</v>
+      </c>
+      <c r="F306" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I306" t="n">
+        <v>0</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0.552210168931135</v>
+      </c>
+      <c r="K306"/>
+      <c r="L306"/>
+      <c r="M306"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="s">
+        <v>31</v>
+      </c>
+      <c r="B307" t="s">
+        <v>29</v>
+      </c>
+      <c r="C307" t="s">
+        <v>23</v>
+      </c>
+      <c r="D307" t="s">
+        <v>16</v>
+      </c>
+      <c r="E307" t="n">
+        <v>14</v>
+      </c>
+      <c r="F307" t="n">
+        <v>5711</v>
+      </c>
+      <c r="G307" t="n">
+        <v>200</v>
+      </c>
+      <c r="H307" t="n">
+        <v>0.270833333333333</v>
+      </c>
+      <c r="I307" t="n">
+        <v>0</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0.552210168931135</v>
+      </c>
+      <c r="K307" t="n">
+        <v>0.567164179104478</v>
+      </c>
+      <c r="L307" t="n">
+        <v>0.348854166666667</v>
+      </c>
+      <c r="M307" t="n">
+        <v>0.261220472211878</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>